<commit_message>
Update Dashboard to display flu data on preview site.
</commit_message>
<xml_diff>
--- a/analysis/resources/WaTCH_Tables.xlsx
+++ b/analysis/resources/WaTCH_Tables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10212"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tpd0001/github/watch-wv/analysis/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCBF2398-40A2-E541-A404-164EB4BB78D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7A1000E-7437-8741-851F-50A471AB1109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="600" yWindow="760" windowWidth="26960" windowHeight="18880" xr2:uid="{ABEE2980-A2EF-284E-9534-8BF6C1D1D8CC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="244">
   <si>
     <t>capacity_mgd</t>
   </si>
@@ -714,9 +714,6 @@
     <t>withdrawn</t>
   </si>
   <si>
-    <t>SR</t>
-  </si>
-  <si>
     <t>Cabell,Wayne</t>
   </si>
   <si>
@@ -742,6 +739,33 @@
   </si>
   <si>
     <t>College Park Apartments</t>
+  </si>
+  <si>
+    <t>SaltRockWWTP</t>
+  </si>
+  <si>
+    <t>BarboursvilleLagoon</t>
+  </si>
+  <si>
+    <t>CharlestonSanitaryBoardWWTP</t>
+  </si>
+  <si>
+    <t>DunbarWWTP</t>
+  </si>
+  <si>
+    <t>HurricaneWWTP</t>
+  </si>
+  <si>
+    <t>HuntingtonSanitaryBoardWWTP</t>
+  </si>
+  <si>
+    <t>PeaRidgeWWTP-C</t>
+  </si>
+  <si>
+    <t>PeaRidgeWWTP-A</t>
+  </si>
+  <si>
+    <t>72-hr time-weighted composite</t>
   </si>
 </sst>
 </file>
@@ -1512,7 +1536,7 @@
         <v>122</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>27</v>
@@ -1674,13 +1698,13 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="41" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>122</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>27</v>
@@ -1725,7 +1749,7 @@
         <v>26505</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
@@ -1881,7 +1905,7 @@
         <v>78</v>
       </c>
       <c r="C11" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D11" t="s">
         <v>27</v>
@@ -3432,10 +3456,10 @@
         <v>38.400744931017101</v>
       </c>
       <c r="J40" t="s">
-        <v>207</v>
+        <v>240</v>
       </c>
       <c r="K40" s="31" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L40" s="34">
         <v>17</v>
@@ -3838,13 +3862,13 @@
     </row>
     <row r="48" spans="1:18" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="19" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>122</v>
       </c>
       <c r="C48" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D48" s="33" t="s">
         <v>26</v>
@@ -3865,10 +3889,10 @@
         <v>38.856708400000002</v>
       </c>
       <c r="J48" t="s">
+        <v>227</v>
+      </c>
+      <c r="K48" t="s">
         <v>228</v>
-      </c>
-      <c r="K48" t="s">
-        <v>229</v>
       </c>
       <c r="L48" s="18">
         <v>0.7</v>
@@ -4393,7 +4417,7 @@
         <v>38.414946823509098</v>
       </c>
       <c r="J58" t="s">
-        <v>209</v>
+        <v>236</v>
       </c>
       <c r="K58" s="31" t="s">
         <v>192</v>
@@ -4449,7 +4473,7 @@
         <v>38.373735533484897</v>
       </c>
       <c r="J59" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="K59" s="31" t="s">
         <v>4</v>
@@ -4502,7 +4526,7 @@
         <v>38.368519014596998</v>
       </c>
       <c r="J60" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="K60" s="31" t="s">
         <v>4</v>
@@ -4555,7 +4579,7 @@
         <v>38.446524084559897</v>
       </c>
       <c r="J61" t="s">
-        <v>207</v>
+        <v>239</v>
       </c>
       <c r="K61" s="31" t="s">
         <v>196</v>
@@ -4570,7 +4594,7 @@
         <v>55486</v>
       </c>
       <c r="O61" s="35" t="s">
-        <v>18</v>
+        <v>243</v>
       </c>
       <c r="P61" s="33" t="s">
         <v>31</v>
@@ -4584,7 +4608,7 @@
         <v>200</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>122</v>
+        <v>78</v>
       </c>
       <c r="C62" s="31" t="s">
         <v>201</v>
@@ -4608,7 +4632,7 @@
         <v>38.343336164586603</v>
       </c>
       <c r="J62" t="s">
-        <v>207</v>
+        <v>240</v>
       </c>
       <c r="K62" s="31" t="s">
         <v>202</v>
@@ -4664,7 +4688,7 @@
         <v>38.572623654172197</v>
       </c>
       <c r="J63" t="s">
-        <v>215</v>
+        <v>241</v>
       </c>
       <c r="K63" s="31" t="s">
         <v>192</v>
@@ -4774,7 +4798,7 @@
         <v>38.419661908139098</v>
       </c>
       <c r="J65" t="s">
-        <v>215</v>
+        <v>242</v>
       </c>
       <c r="K65" s="31" t="s">
         <v>192</v>
@@ -4821,22 +4845,22 @@
         <v>178</v>
       </c>
       <c r="H66" s="31">
-        <v>-82.209446953848399</v>
+        <v>-82.105144999999993</v>
       </c>
       <c r="I66" s="31">
-        <v>38.431960787764801</v>
+        <v>38.425437000000002</v>
       </c>
       <c r="J66" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="K66" s="31" t="s">
         <v>192</v>
       </c>
       <c r="L66" s="34">
-        <v>2.5</v>
+        <v>1.8</v>
       </c>
       <c r="M66" s="34">
-        <v>11250</v>
+        <v>7200</v>
       </c>
       <c r="N66" s="40">
         <v>96319</v>
@@ -4848,7 +4872,7 @@
         <v>31</v>
       </c>
       <c r="Q66" s="32">
-        <v>25545</v>
+        <v>25541</v>
       </c>
       <c r="R66" s="31" t="s">
         <v>197</v>
@@ -4877,22 +4901,22 @@
         <v>178</v>
       </c>
       <c r="H67" s="31">
-        <v>-82.209446953848399</v>
+        <v>-82.244877751268803</v>
       </c>
       <c r="I67" s="31">
-        <v>38.431960787764801</v>
+        <v>38.372162360135</v>
       </c>
       <c r="J67" t="s">
-        <v>226</v>
+        <v>235</v>
       </c>
       <c r="K67" s="31" t="s">
         <v>192</v>
       </c>
       <c r="L67" s="34">
-        <v>2.5</v>
+        <v>0.7</v>
       </c>
       <c r="M67" s="34">
-        <v>11250</v>
+        <v>4050</v>
       </c>
       <c r="N67" s="40">
         <v>96319</v>

</xml_diff>